<commit_message>
Update to API Calls, Update Query and response structure
</commit_message>
<xml_diff>
--- a/manitoba_childcare.xlsx
+++ b/manitoba_childcare.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,8 +70,12 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +90,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +136,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:AD26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -501,25 +516,30 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="55" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="55" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -560,104 +580,2357 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Province</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Postal Code</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Neighbourhood</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Infant (0–2) Vacancies</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Preschool (2–6) Vacancies</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Nursery (2–6) Vacancies</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>School Age (6–12) Vacancies</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Open Weekdays</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Open Weekends</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Open Evenings</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Open Overnight</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Employment Opportunities</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Profile URL</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Scraped At</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Total facilities: 0</t>
-        </is>
-      </c>
-      <c r="Y2" s="8" t="inlineStr">
-        <is>
-          <t>Last scraped: 2026-06-06 23:39</t>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="9" t="inlineStr"/>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>&amp;quot;Bundles of Joyce&amp;quot; - Jaimie Joyce</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="inlineStr"/>
+      <c r="J2" s="9" t="inlineStr"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'ce4d36cb-7c96-4b9e-bcdc-b268f9c36b87', 'name': 'EASTMAN'}</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': 'a076deac-718c-412b-b44d-06a2bef4cb3f', 'name': 'EASTMAN'}</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': 'f62e758d-6eb4-415d-a17c-dd48fb5c1410', 'name': 'STE. ANNE'}</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>(204) 346-4333</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>jaimie.helgason@gmail.com</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr"/>
+      <c r="Q2" s="9" t="inlineStr"/>
+      <c r="R2" s="9" t="inlineStr"/>
+      <c r="S2" s="9" t="inlineStr"/>
+      <c r="T2" s="9" t="inlineStr"/>
+      <c r="U2" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V2" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W2" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X2" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y2" s="9" t="inlineStr"/>
+      <c r="Z2" s="9" t="inlineStr"/>
+      <c r="AA2" s="9" t="inlineStr">
+        <is>
+          <t>49.66806</t>
+        </is>
+      </c>
+      <c r="AB2" s="9" t="inlineStr">
+        <is>
+          <t>-96.66392</t>
+        </is>
+      </c>
+      <c r="AC2" s="9" t="inlineStr"/>
+      <c r="AD2" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="10" t="inlineStr"/>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>(Gi) Kinaa'amaadiiwigamingoons Little Teaching Lodge Aboriginal Head Start</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'c856898a-6f6c-476c-9691-2212b4ac8772', 'type': 'NURSERY'}</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr"/>
+      <c r="G3" s="10" t="inlineStr"/>
+      <c r="H3" s="10" t="inlineStr"/>
+      <c r="I3" s="10" t="inlineStr"/>
+      <c r="J3" s="10" t="inlineStr"/>
+      <c r="K3" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': '657be827-354f-45f9-a14f-05d849912a73', 'name': 'WESTMAN'}</t>
+        </is>
+      </c>
+      <c r="L3" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': '5b786b20-95ee-4993-a09c-56752b9c0c52', 'name': 'BRANDON'}</t>
+        </is>
+      </c>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '0b391143-9c68-4f99-8a0c-e5bd858e8257', 'name': 'BRANDON EAST'}</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
+          <t>(204) 729-0788</t>
+        </is>
+      </c>
+      <c r="O3" s="10" t="inlineStr">
+        <is>
+          <t>ltglodge@mymts.net</t>
+        </is>
+      </c>
+      <c r="P3" s="10" t="inlineStr"/>
+      <c r="Q3" s="10" t="inlineStr"/>
+      <c r="R3" s="10" t="inlineStr"/>
+      <c r="S3" s="10" t="inlineStr"/>
+      <c r="T3" s="10" t="inlineStr"/>
+      <c r="U3" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V3" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W3" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X3" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y3" s="10" t="inlineStr"/>
+      <c r="Z3" s="10" t="inlineStr"/>
+      <c r="AA3" s="10" t="inlineStr">
+        <is>
+          <t>49.837932</t>
+        </is>
+      </c>
+      <c r="AB3" s="10" t="inlineStr">
+        <is>
+          <t>-99.940841</t>
+        </is>
+      </c>
+      <c r="AC3" s="10" t="inlineStr"/>
+      <c r="AD3" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="9" t="inlineStr"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>3 Little Kittens Home Daycare</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="9" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr"/>
+      <c r="I4" s="9" t="inlineStr"/>
+      <c r="J4" s="9" t="inlineStr"/>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '5d7a163d-1550-44b5-8f2b-8e552700dcf6', 'name': 'SEVEN OAKS'}</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '4d9a0938-4e7a-4398-80d0-2b9b780f8320', 'name': 'MANDALAY WEST'}</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr"/>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>3littlekittens@outlook.com</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr"/>
+      <c r="Q4" s="9" t="inlineStr"/>
+      <c r="R4" s="9" t="inlineStr"/>
+      <c r="S4" s="9" t="inlineStr"/>
+      <c r="T4" s="9" t="inlineStr"/>
+      <c r="U4" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V4" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W4" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X4" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y4" s="9" t="inlineStr"/>
+      <c r="Z4" s="9" t="inlineStr"/>
+      <c r="AA4" s="9" t="inlineStr">
+        <is>
+          <t>49.967259</t>
+        </is>
+      </c>
+      <c r="AB4" s="9" t="inlineStr">
+        <is>
+          <t>-97.174314</t>
+        </is>
+      </c>
+      <c r="AC4" s="9" t="inlineStr"/>
+      <c r="AD4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="10" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>A to Z Child Care</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': 'cd719f83-60de-4613-b06e-0a1d25a86628', 'type': 'Non Funded'}</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr"/>
+      <c r="H5" s="10" t="inlineStr"/>
+      <c r="I5" s="10" t="inlineStr"/>
+      <c r="J5" s="10" t="inlineStr"/>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'ce4d36cb-7c96-4b9e-bcdc-b268f9c36b87', 'name': 'EASTMAN'}</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'a076deac-718c-412b-b44d-06a2bef4cb3f', 'name': 'EASTMAN'}</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': 'cbb928d6-94e6-4b30-8e4a-133677a514a3', 'name': 'STEINBACH'}</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr"/>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>Atozchildcare2020@gmail.com</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr"/>
+      <c r="Q5" s="10" t="inlineStr"/>
+      <c r="R5" s="10" t="inlineStr"/>
+      <c r="S5" s="10" t="inlineStr"/>
+      <c r="T5" s="10" t="inlineStr"/>
+      <c r="U5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X5" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y5" s="10" t="inlineStr"/>
+      <c r="Z5" s="10" t="inlineStr"/>
+      <c r="AA5" s="10" t="inlineStr">
+        <is>
+          <t>49.59127</t>
+        </is>
+      </c>
+      <c r="AB5" s="10" t="inlineStr">
+        <is>
+          <t>-96.890882</t>
+        </is>
+      </c>
+      <c r="AC5" s="10" t="inlineStr"/>
+      <c r="AD5" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="9" t="inlineStr"/>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Abi Family Childcare</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr"/>
+      <c r="J6" s="9" t="inlineStr"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '3f9c038f-f217-405c-9429-c6cfabd900ed', 'name': 'ST. BONIFACE'}</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '5ee12b52-03c1-4d4e-bb20-c0a38243fa0c', 'name': 'ISLAND LAKES'}</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr"/>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>Abi4childcare@gmail.com</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr"/>
+      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="R6" s="9" t="inlineStr"/>
+      <c r="S6" s="9" t="inlineStr"/>
+      <c r="T6" s="9" t="inlineStr"/>
+      <c r="U6" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V6" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W6" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X6" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y6" s="9" t="inlineStr"/>
+      <c r="Z6" s="9" t="inlineStr"/>
+      <c r="AA6" s="9" t="inlineStr">
+        <is>
+          <t>53.760861</t>
+        </is>
+      </c>
+      <c r="AB6" s="9" t="inlineStr">
+        <is>
+          <t>-98.813876</t>
+        </is>
+      </c>
+      <c r="AC6" s="9" t="inlineStr"/>
+      <c r="AD6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Abiodun Akinlosotu</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="10" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'f2b3e384-0b70-44be-bd32-7509c93bd993', 'name': 'FORT GARRY'}</t>
+        </is>
+      </c>
+      <c r="M7" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': 'ab550ec5-2d4f-4bae-9ec1-53e5abd1b6dc', 'name': 'MAYBANK'}</t>
+        </is>
+      </c>
+      <c r="N7" s="10" t="inlineStr"/>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>gladtidingsdaycare@gmail.com</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="inlineStr"/>
+      <c r="Q7" s="10" t="inlineStr"/>
+      <c r="R7" s="10" t="inlineStr"/>
+      <c r="S7" s="10" t="inlineStr"/>
+      <c r="T7" s="10" t="inlineStr"/>
+      <c r="U7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X7" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y7" s="10" t="inlineStr"/>
+      <c r="Z7" s="10" t="inlineStr"/>
+      <c r="AA7" s="10" t="inlineStr">
+        <is>
+          <t>49.833662</t>
+        </is>
+      </c>
+      <c r="AB7" s="10" t="inlineStr">
+        <is>
+          <t>-97.155858</t>
+        </is>
+      </c>
+      <c r="AC7" s="10" t="inlineStr"/>
+      <c r="AD7" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="9" t="inlineStr"/>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Abiola Eseyin</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr"/>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '3f9c038f-f217-405c-9429-c6cfabd900ed', 'name': 'ST. BONIFACE'}</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '5ee12b52-03c1-4d4e-bb20-c0a38243fa0c', 'name': 'ISLAND LAKES'}</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr"/>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>giggleshomedaycare@outlook.com</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr"/>
+      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="R8" s="9" t="inlineStr"/>
+      <c r="S8" s="9" t="inlineStr"/>
+      <c r="T8" s="9" t="inlineStr"/>
+      <c r="U8" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V8" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W8" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X8" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y8" s="9" t="inlineStr"/>
+      <c r="Z8" s="9" t="inlineStr"/>
+      <c r="AA8" s="9" t="inlineStr">
+        <is>
+          <t>49.821701</t>
+        </is>
+      </c>
+      <c r="AB8" s="9" t="inlineStr">
+        <is>
+          <t>-97.058624</t>
+        </is>
+      </c>
+      <c r="AC8" s="9" t="inlineStr"/>
+      <c r="AD8" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="10" t="inlineStr"/>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Acorn Family Place Playroom</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'c856898a-6f6c-476c-9691-2212b4ac8772', 'type': 'NURSERY'}</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr"/>
+      <c r="G9" s="10" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr"/>
+      <c r="I9" s="10" t="inlineStr"/>
+      <c r="J9" s="10" t="inlineStr"/>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'b9a5c232-da2a-41ef-a8ec-2ae646846a44', 'name': 'DOWNTOWN'}</t>
+        </is>
+      </c>
+      <c r="M9" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '39cf7e92-956a-40c0-8b1f-c264e2fcdbfa', 'name': 'WEST BROADWAY'}</t>
+        </is>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>(204) 560-3151</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>playroom@acornfamilyplace.ca</t>
+        </is>
+      </c>
+      <c r="P9" s="10" t="inlineStr"/>
+      <c r="Q9" s="10" t="inlineStr"/>
+      <c r="R9" s="10" t="inlineStr"/>
+      <c r="S9" s="10" t="inlineStr"/>
+      <c r="T9" s="10" t="inlineStr"/>
+      <c r="U9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X9" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y9" s="10" t="inlineStr"/>
+      <c r="Z9" s="10" t="inlineStr"/>
+      <c r="AA9" s="10" t="inlineStr">
+        <is>
+          <t>49.885969</t>
+        </is>
+      </c>
+      <c r="AB9" s="10" t="inlineStr">
+        <is>
+          <t>-97.157868</t>
+        </is>
+      </c>
+      <c r="AC9" s="10" t="inlineStr"/>
+      <c r="AD9" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="9" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Action Centre Day Nursery Inc.</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr"/>
+      <c r="I10" s="9" t="inlineStr"/>
+      <c r="J10" s="9" t="inlineStr"/>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '1f924ce1-0342-46a1-946d-05cc169d230f', 'name': 'POINT DOUGLAS'}</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '22b8b1c0-9115-4ad9-bc40-dc9402d9155a', 'name': 'LORD SELKIRK PARK'}</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr"/>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>actioncentredaynursery1974@gmail.com</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr"/>
+      <c r="Q10" s="9" t="inlineStr"/>
+      <c r="R10" s="9" t="inlineStr"/>
+      <c r="S10" s="9" t="inlineStr"/>
+      <c r="T10" s="9" t="inlineStr"/>
+      <c r="U10" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V10" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W10" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X10" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y10" s="9" t="inlineStr"/>
+      <c r="Z10" s="9" t="inlineStr"/>
+      <c r="AA10" s="9" t="inlineStr">
+        <is>
+          <t>49.911647</t>
+        </is>
+      </c>
+      <c r="AB10" s="9" t="inlineStr">
+        <is>
+          <t>-97.141671</t>
+        </is>
+      </c>
+      <c r="AC10" s="9" t="inlineStr"/>
+      <c r="AD10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Adelle Kennedy</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': 'cd719f83-60de-4613-b06e-0a1d25a86628', 'type': 'Non Funded'}</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr"/>
+      <c r="G11" s="10" t="inlineStr"/>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="10" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'f2b3e384-0b70-44be-bd32-7509c93bd993', 'name': 'FORT GARRY'}</t>
+        </is>
+      </c>
+      <c r="M11" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '8ff2793f-f602-4212-b307-6fe8ce8b628d', 'name': 'FORT RICHMOND'}</t>
+        </is>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>(204) 269-0183</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="inlineStr"/>
+      <c r="P11" s="10" t="inlineStr"/>
+      <c r="Q11" s="10" t="inlineStr"/>
+      <c r="R11" s="10" t="inlineStr"/>
+      <c r="S11" s="10" t="inlineStr"/>
+      <c r="T11" s="10" t="inlineStr"/>
+      <c r="U11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X11" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y11" s="10" t="inlineStr"/>
+      <c r="Z11" s="10" t="inlineStr"/>
+      <c r="AA11" s="10" t="inlineStr">
+        <is>
+          <t>49.795892</t>
+        </is>
+      </c>
+      <c r="AB11" s="10" t="inlineStr">
+        <is>
+          <t>-97.14008</t>
+        </is>
+      </c>
+      <c r="AC11" s="10" t="inlineStr"/>
+      <c r="AD11" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="9" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Adorable Child Care</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr"/>
+      <c r="J12" s="9" t="inlineStr"/>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': 'f2b3e384-0b70-44be-bd32-7509c93bd993', 'name': 'FORT GARRY'}</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '792b81b8-bb44-4998-8872-f22cbab32883', 'name': 'WAVERLEY WEST'}</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr"/>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>adorable4family@gmail.com</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr"/>
+      <c r="Q12" s="9" t="inlineStr"/>
+      <c r="R12" s="9" t="inlineStr"/>
+      <c r="S12" s="9" t="inlineStr"/>
+      <c r="T12" s="9" t="inlineStr"/>
+      <c r="U12" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V12" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W12" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X12" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y12" s="9" t="inlineStr"/>
+      <c r="Z12" s="9" t="inlineStr"/>
+      <c r="AA12" s="9" t="inlineStr">
+        <is>
+          <t>49.773981</t>
+        </is>
+      </c>
+      <c r="AB12" s="9" t="inlineStr">
+        <is>
+          <t>-97.182246</t>
+        </is>
+      </c>
+      <c r="AC12" s="9" t="inlineStr"/>
+      <c r="AD12" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="10" t="inlineStr"/>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Adrielle Steppler</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': 'cd719f83-60de-4613-b06e-0a1d25a86628', 'type': 'Non Funded'}</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr"/>
+      <c r="G13" s="10" t="inlineStr"/>
+      <c r="H13" s="10" t="inlineStr"/>
+      <c r="I13" s="10" t="inlineStr"/>
+      <c r="J13" s="10" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': '3afcd904-dbb6-4a31-bb58-98c639233033', 'name': 'CENTRAL'}</t>
+        </is>
+      </c>
+      <c r="L13" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'ddc8b400-ad11-4fd6-a9dd-0582811d84d9', 'name': 'CENTRAL'}</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '94571598-be96-4d6f-9543-671c4cdf65b4', 'name': 'PORTAGE LA PRAIRIE'}</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="inlineStr"/>
+      <c r="O13" s="10" t="inlineStr">
+        <is>
+          <t>adriellekroeker@gmail.com</t>
+        </is>
+      </c>
+      <c r="P13" s="10" t="inlineStr"/>
+      <c r="Q13" s="10" t="inlineStr"/>
+      <c r="R13" s="10" t="inlineStr"/>
+      <c r="S13" s="10" t="inlineStr"/>
+      <c r="T13" s="10" t="inlineStr"/>
+      <c r="U13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X13" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y13" s="10" t="inlineStr"/>
+      <c r="Z13" s="10" t="inlineStr"/>
+      <c r="AA13" s="10" t="inlineStr">
+        <is>
+          <t>49.967895</t>
+        </is>
+      </c>
+      <c r="AB13" s="10" t="inlineStr">
+        <is>
+          <t>-98.28527</t>
+        </is>
+      </c>
+      <c r="AC13" s="10" t="inlineStr"/>
+      <c r="AD13" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="9" t="inlineStr"/>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Advantage Child Care Academy - McGillivray</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': 'cd719f83-60de-4613-b06e-0a1d25a86628', 'type': 'Non Funded'}</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr"/>
+      <c r="J14" s="9" t="inlineStr"/>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': '3afcd904-dbb6-4a31-bb58-98c639233033', 'name': 'CENTRAL'}</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': 'ddc8b400-ad11-4fd6-a9dd-0582811d84d9', 'name': 'CENTRAL'}</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': 'e3a6c0e7-3b38-4494-910f-8820cc62d367', 'name': 'OAK BLUFF'}</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="inlineStr"/>
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>hdhanjal@advantagechildcareacademy.ca</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr"/>
+      <c r="Q14" s="9" t="inlineStr"/>
+      <c r="R14" s="9" t="inlineStr"/>
+      <c r="S14" s="9" t="inlineStr"/>
+      <c r="T14" s="9" t="inlineStr"/>
+      <c r="U14" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V14" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W14" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X14" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y14" s="9" t="inlineStr"/>
+      <c r="Z14" s="9" t="inlineStr"/>
+      <c r="AA14" s="9" t="inlineStr">
+        <is>
+          <t>49.803633</t>
+        </is>
+      </c>
+      <c r="AB14" s="9" t="inlineStr">
+        <is>
+          <t>-97.237816</t>
+        </is>
+      </c>
+      <c r="AC14" s="9" t="inlineStr"/>
+      <c r="AD14" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Advantage Child Care Academy Inc.</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': 'cd719f83-60de-4613-b06e-0a1d25a86628', 'type': 'Non Funded'}</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="10" t="inlineStr"/>
+      <c r="I15" s="10" t="inlineStr"/>
+      <c r="J15" s="10" t="inlineStr"/>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L15" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'f2b3e384-0b70-44be-bd32-7509c93bd993', 'name': 'FORT GARRY'}</t>
+        </is>
+      </c>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '6f928855-eed0-4250-bdcb-3ab805fd3008', 'name': 'WEST FORT GARRY INDUSTRIAL'}</t>
+        </is>
+      </c>
+      <c r="N15" s="10" t="inlineStr"/>
+      <c r="O15" s="10" t="inlineStr">
+        <is>
+          <t>hdhanjal@advantagechildcareacademy.ca</t>
+        </is>
+      </c>
+      <c r="P15" s="10" t="inlineStr"/>
+      <c r="Q15" s="10" t="inlineStr"/>
+      <c r="R15" s="10" t="inlineStr"/>
+      <c r="S15" s="10" t="inlineStr"/>
+      <c r="T15" s="10" t="inlineStr"/>
+      <c r="U15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X15" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y15" s="10" t="inlineStr"/>
+      <c r="Z15" s="10" t="inlineStr"/>
+      <c r="AA15" s="10" t="inlineStr">
+        <is>
+          <t>49.818503</t>
+        </is>
+      </c>
+      <c r="AB15" s="10" t="inlineStr">
+        <is>
+          <t>-97.186041</t>
+        </is>
+      </c>
+      <c r="AC15" s="10" t="inlineStr"/>
+      <c r="AD15" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="9" t="inlineStr"/>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Afshan Noreen</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="9" t="inlineStr"/>
+      <c r="H16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="inlineStr"/>
+      <c r="J16" s="9" t="inlineStr"/>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '3f9c038f-f217-405c-9429-c6cfabd900ed', 'name': 'ST. BONIFACE'}</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '9f34d0d5-f6ba-4f52-8645-7f3f05460ea1', 'name': 'ROYALWOOD'}</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>(431) 999-8974</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr"/>
+      <c r="P16" s="9" t="inlineStr"/>
+      <c r="Q16" s="9" t="inlineStr"/>
+      <c r="R16" s="9" t="inlineStr"/>
+      <c r="S16" s="9" t="inlineStr"/>
+      <c r="T16" s="9" t="inlineStr"/>
+      <c r="U16" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V16" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W16" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X16" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y16" s="9" t="inlineStr"/>
+      <c r="Z16" s="9" t="inlineStr"/>
+      <c r="AA16" s="9" t="inlineStr">
+        <is>
+          <t>49.819972</t>
+        </is>
+      </c>
+      <c r="AB16" s="9" t="inlineStr">
+        <is>
+          <t>-97.073086</t>
+        </is>
+      </c>
+      <c r="AC16" s="9" t="inlineStr"/>
+      <c r="AD16" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="10" t="inlineStr"/>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Agassiz Child Care Centre Inc.</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
+      <c r="I17" s="10" t="inlineStr"/>
+      <c r="J17" s="10" t="inlineStr"/>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L17" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'f2b3e384-0b70-44be-bd32-7509c93bd993', 'name': 'FORT GARRY'}</t>
+        </is>
+      </c>
+      <c r="M17" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '8ff2793f-f602-4212-b307-6fe8ce8b628d', 'name': 'FORT RICHMOND'}</t>
+        </is>
+      </c>
+      <c r="N17" s="10" t="inlineStr">
+        <is>
+          <t>(204) 269-3779</t>
+        </is>
+      </c>
+      <c r="O17" s="10" t="inlineStr">
+        <is>
+          <t>agassizchildcare@gmail.com</t>
+        </is>
+      </c>
+      <c r="P17" s="10" t="inlineStr"/>
+      <c r="Q17" s="10" t="inlineStr"/>
+      <c r="R17" s="10" t="inlineStr"/>
+      <c r="S17" s="10" t="inlineStr"/>
+      <c r="T17" s="10" t="inlineStr"/>
+      <c r="U17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X17" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y17" s="10" t="inlineStr"/>
+      <c r="Z17" s="10" t="inlineStr"/>
+      <c r="AA17" s="10" t="inlineStr">
+        <is>
+          <t>49.799534</t>
+        </is>
+      </c>
+      <c r="AB17" s="10" t="inlineStr">
+        <is>
+          <t>-97.13459</t>
+        </is>
+      </c>
+      <c r="AC17" s="10" t="inlineStr"/>
+      <c r="AD17" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="9" t="inlineStr"/>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Home Based Child Care</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="9" t="inlineStr"/>
+      <c r="H18" s="9" t="inlineStr"/>
+      <c r="I18" s="9" t="inlineStr"/>
+      <c r="J18" s="9" t="inlineStr"/>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': '3afcd904-dbb6-4a31-bb58-98c639233033', 'name': 'CENTRAL'}</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': 'ddc8b400-ad11-4fd6-a9dd-0582811d84d9', 'name': 'CENTRAL'}</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '1d52ed96-0e50-4c20-9832-41852d753966', 'name': 'ALTONA'}</t>
+        </is>
+      </c>
+      <c r="N18" s="9" t="inlineStr"/>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>5thavenuefcc@gmail.com</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr"/>
+      <c r="Q18" s="9" t="inlineStr"/>
+      <c r="R18" s="9" t="inlineStr"/>
+      <c r="S18" s="9" t="inlineStr"/>
+      <c r="T18" s="9" t="inlineStr"/>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V18" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X18" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y18" s="9" t="inlineStr"/>
+      <c r="Z18" s="9" t="inlineStr"/>
+      <c r="AA18" s="9" t="inlineStr">
+        <is>
+          <t>49.074793</t>
+        </is>
+      </c>
+      <c r="AB18" s="9" t="inlineStr">
+        <is>
+          <t>-95.644772</t>
+        </is>
+      </c>
+      <c r="AC18" s="9" t="inlineStr"/>
+      <c r="AD18" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="10" t="inlineStr"/>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Aleph-Bet Child Life Enrichment Forest Park School Age Program Inc.</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr"/>
+      <c r="G19" s="10" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr"/>
+      <c r="I19" s="10" t="inlineStr"/>
+      <c r="J19" s="10" t="inlineStr"/>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L19" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': '5d7a163d-1550-44b5-8f2b-8e552700dcf6', 'name': 'SEVEN OAKS'}</t>
+        </is>
+      </c>
+      <c r="M19" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '69824b53-25e0-4a24-8d32-5f92814b12fa', 'name': 'GARDEN CITY'}</t>
+        </is>
+      </c>
+      <c r="N19" s="10" t="inlineStr"/>
+      <c r="O19" s="10" t="inlineStr">
+        <is>
+          <t>robyn@alephbet.ca</t>
+        </is>
+      </c>
+      <c r="P19" s="10" t="inlineStr"/>
+      <c r="Q19" s="10" t="inlineStr"/>
+      <c r="R19" s="10" t="inlineStr"/>
+      <c r="S19" s="10" t="inlineStr"/>
+      <c r="T19" s="10" t="inlineStr"/>
+      <c r="U19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X19" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y19" s="10" t="inlineStr"/>
+      <c r="Z19" s="10" t="inlineStr"/>
+      <c r="AA19" s="10" t="inlineStr">
+        <is>
+          <t>49.944062</t>
+        </is>
+      </c>
+      <c r="AB19" s="10" t="inlineStr">
+        <is>
+          <t>-97.138356</t>
+        </is>
+      </c>
+      <c r="AC19" s="10" t="inlineStr"/>
+      <c r="AD19" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="9" t="inlineStr"/>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Aleph-Bet Child Life Enrichment Program Inc.</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="9" t="inlineStr"/>
+      <c r="H20" s="9" t="inlineStr"/>
+      <c r="I20" s="9" t="inlineStr"/>
+      <c r="J20" s="9" t="inlineStr"/>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '5d7a163d-1550-44b5-8f2b-8e552700dcf6', 'name': 'SEVEN OAKS'}</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '69824b53-25e0-4a24-8d32-5f92814b12fa', 'name': 'GARDEN CITY'}</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr"/>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>robyn@alephbet.ca</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr"/>
+      <c r="Q20" s="9" t="inlineStr"/>
+      <c r="R20" s="9" t="inlineStr"/>
+      <c r="S20" s="9" t="inlineStr"/>
+      <c r="T20" s="9" t="inlineStr"/>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V20" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W20" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X20" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y20" s="9" t="inlineStr"/>
+      <c r="Z20" s="9" t="inlineStr"/>
+      <c r="AA20" s="9" t="inlineStr">
+        <is>
+          <t>49.9474</t>
+        </is>
+      </c>
+      <c r="AB20" s="9" t="inlineStr">
+        <is>
+          <t>-97.136531</t>
+        </is>
+      </c>
+      <c r="AC20" s="9" t="inlineStr"/>
+      <c r="AD20" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Aleph-Bet Child Life Enrichment School Age Program Inc. - Margaret Park</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'da9a9b8c-d169-4c2b-8886-1d6078970bf8', 'type': 'CENTRE'}</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr"/>
+      <c r="G21" s="10" t="inlineStr"/>
+      <c r="H21" s="10" t="inlineStr"/>
+      <c r="I21" s="10" t="inlineStr"/>
+      <c r="J21" s="10" t="inlineStr"/>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': '5d7a163d-1550-44b5-8f2b-8e552700dcf6', 'name': 'SEVEN OAKS'}</t>
+        </is>
+      </c>
+      <c r="M21" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '69824b53-25e0-4a24-8d32-5f92814b12fa', 'name': 'GARDEN CITY'}</t>
+        </is>
+      </c>
+      <c r="N21" s="10" t="inlineStr"/>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>robyn@alephbet.ca</t>
+        </is>
+      </c>
+      <c r="P21" s="10" t="inlineStr"/>
+      <c r="Q21" s="10" t="inlineStr"/>
+      <c r="R21" s="10" t="inlineStr"/>
+      <c r="S21" s="10" t="inlineStr"/>
+      <c r="T21" s="10" t="inlineStr"/>
+      <c r="U21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y21" s="10" t="inlineStr"/>
+      <c r="Z21" s="10" t="inlineStr"/>
+      <c r="AA21" s="10" t="inlineStr">
+        <is>
+          <t>49.947902</t>
+        </is>
+      </c>
+      <c r="AB21" s="10" t="inlineStr">
+        <is>
+          <t>-97.120846</t>
+        </is>
+      </c>
+      <c r="AC21" s="10" t="inlineStr"/>
+      <c r="AD21" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr"/>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Alice Ando Goli</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="9" t="inlineStr"/>
+      <c r="H22" s="9" t="inlineStr"/>
+      <c r="I22" s="9" t="inlineStr"/>
+      <c r="J22" s="9" t="inlineStr"/>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '3f9c038f-f217-405c-9429-c6cfabd900ed', 'name': 'ST. BONIFACE'}</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '8d5ce148-9835-4d6d-9afd-3728aabe6b3d', 'name': 'SAGE CREEK'}</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr"/>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>alicenestcare@outlook.com</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr"/>
+      <c r="Q22" s="9" t="inlineStr"/>
+      <c r="R22" s="9" t="inlineStr"/>
+      <c r="S22" s="9" t="inlineStr"/>
+      <c r="T22" s="9" t="inlineStr"/>
+      <c r="U22" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V22" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W22" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X22" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y22" s="9" t="inlineStr"/>
+      <c r="Z22" s="9" t="inlineStr"/>
+      <c r="AA22" s="9" t="inlineStr">
+        <is>
+          <t>49.839952</t>
+        </is>
+      </c>
+      <c r="AB22" s="9" t="inlineStr">
+        <is>
+          <t>-97.032497</t>
+        </is>
+      </c>
+      <c r="AC22" s="9" t="inlineStr"/>
+      <c r="AD22" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="10" t="inlineStr"/>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Alma Rongcal</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr"/>
+      <c r="G23" s="10" t="inlineStr"/>
+      <c r="H23" s="10" t="inlineStr"/>
+      <c r="I23" s="10" t="inlineStr"/>
+      <c r="J23" s="10" t="inlineStr"/>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'db995ee7-0028-44a3-a93a-ff26e53af0ac', 'name': 'ST. JAMES ASSINIBOINE'}</t>
+        </is>
+      </c>
+      <c r="M23" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '2805185d-8254-46cd-a6a5-2636f0c5611b', 'name': 'HERITAGE PARK'}</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr"/>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>almarongcal@yahoo.com</t>
+        </is>
+      </c>
+      <c r="P23" s="10" t="inlineStr"/>
+      <c r="Q23" s="10" t="inlineStr"/>
+      <c r="R23" s="10" t="inlineStr"/>
+      <c r="S23" s="10" t="inlineStr"/>
+      <c r="T23" s="10" t="inlineStr"/>
+      <c r="U23" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V23" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W23" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X23" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y23" s="10" t="inlineStr"/>
+      <c r="Z23" s="10" t="inlineStr"/>
+      <c r="AA23" s="10" t="inlineStr">
+        <is>
+          <t>49.889716</t>
+        </is>
+      </c>
+      <c r="AB23" s="10" t="inlineStr">
+        <is>
+          <t>-97.283816</t>
+        </is>
+      </c>
+      <c r="AC23" s="10" t="inlineStr"/>
+      <c r="AD23" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="9" t="inlineStr"/>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Almost Home Daycare</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'fe4bc755-6855-42a7-afab-64d1333dd497', 'type': 'HOME'}</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': '1e97be06-3418-4bbc-888b-dedc17c6b078', 'type': 'For-Profit'}</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="9" t="inlineStr"/>
+      <c r="H24" s="9" t="inlineStr"/>
+      <c r="I24" s="9" t="inlineStr"/>
+      <c r="J24" s="9" t="inlineStr"/>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>{'regionId': 'e9f9acf3-ac7b-42a5-8da0-705220851053', 'name': 'WINNIPEG'}</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>{'areaId': '1d417911-afb8-4ccd-922c-3062443bd5eb', 'name': 'TRANSCONA'}</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '6c373a73-15c0-44a4-965e-d45726066ed7', 'name': 'MELROSE'}</t>
+        </is>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
+          <t>(204) 915-5640</t>
+        </is>
+      </c>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>deleon.rachelle@rocketmail.com</t>
+        </is>
+      </c>
+      <c r="P24" s="9" t="inlineStr"/>
+      <c r="Q24" s="9" t="inlineStr"/>
+      <c r="R24" s="9" t="inlineStr"/>
+      <c r="S24" s="9" t="inlineStr"/>
+      <c r="T24" s="9" t="inlineStr"/>
+      <c r="U24" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V24" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W24" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X24" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y24" s="9" t="inlineStr"/>
+      <c r="Z24" s="9" t="inlineStr"/>
+      <c r="AA24" s="9" t="inlineStr">
+        <is>
+          <t>49.894937</t>
+        </is>
+      </c>
+      <c r="AB24" s="9" t="inlineStr">
+        <is>
+          <t>-97.017957</t>
+        </is>
+      </c>
+      <c r="AC24" s="9" t="inlineStr"/>
+      <c r="AD24" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Alonsa Nursery School</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>{'facilityTypeId': 'c856898a-6f6c-476c-9691-2212b4ac8772', 'type': 'NURSERY'}</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>{'businessTypeId': 'c25b2dbe-c4fc-4f04-acd4-e75509cc4f2d', 'type': 'Non-Profit'}</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>{'fundingTypeId': '94f68b71-65da-487f-92c2-21461e0d788b', 'type': 'Funded'}</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="10" t="inlineStr"/>
+      <c r="J25" s="10" t="inlineStr"/>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>{'regionId': '23afdf1c-9109-4029-8ae7-0eb0f26443d2', 'name': 'PARKLAND'}</t>
+        </is>
+      </c>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>{'areaId': 'c15802e6-ba55-4f9b-912c-a359fd273897', 'name': 'PARKLAND'}</t>
+        </is>
+      </c>
+      <c r="M25" s="10" t="inlineStr">
+        <is>
+          <t>{'neighbourhoodId': '3f84b5ac-3df5-4217-90e5-40934b716f50', 'name': 'ALONSA'}</t>
+        </is>
+      </c>
+      <c r="N25" s="10" t="inlineStr"/>
+      <c r="O25" s="10" t="inlineStr">
+        <is>
+          <t>alonsanursery@outlook.com</t>
+        </is>
+      </c>
+      <c r="P25" s="10" t="inlineStr"/>
+      <c r="Q25" s="10" t="inlineStr"/>
+      <c r="R25" s="10" t="inlineStr"/>
+      <c r="S25" s="10" t="inlineStr"/>
+      <c r="T25" s="10" t="inlineStr"/>
+      <c r="U25" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V25" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W25" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="X25" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Y25" s="10" t="inlineStr"/>
+      <c r="Z25" s="10" t="inlineStr"/>
+      <c r="AA25" s="10" t="inlineStr">
+        <is>
+          <t>50.801177</t>
+        </is>
+      </c>
+      <c r="AB25" s="10" t="inlineStr">
+        <is>
+          <t>-98.977607</t>
+        </is>
+      </c>
+      <c r="AC25" s="10" t="inlineStr"/>
+      <c r="AD25" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Total facilities: 24</t>
+        </is>
+      </c>
+      <c r="AD26" s="8" t="inlineStr">
+        <is>
+          <t>Last scraped: 2026-06-07 00:01</t>
         </is>
       </c>
     </row>

</xml_diff>